<commit_message>
docs: fix plan and hardware links, remove duplicate guide and change plan
Align the reading plan with block order and the 30 December 2026 target, and list the plan files in the repository map.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/networking_reading_plan.xlsx
+++ b/docs/networking_reading_plan.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Books" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Reading plan'!$A$8:$G$24</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Reading plan'!$A$8:$F$24</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -66,7 +66,7 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 1 — workload</t>
+    <t xml:space="preserve">Block 1 — workload</t>
   </si>
   <si>
     <t xml:space="preserve">12–18 Oct</t>
@@ -84,7 +84,7 @@
     <t xml:space="preserve">Not read</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 2 — Docker networking</t>
+    <t xml:space="preserve">Block 2 — Docker networking</t>
   </si>
   <si>
     <t xml:space="preserve">19–25 Oct</t>
@@ -135,7 +135,7 @@
     <t xml:space="preserve">If you read only one section, make it this one: a single request through DHCP, DNS, ARP, TCP and HTTP — the ten-questions method told as a story.</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 3 — Linux primitives</t>
+    <t xml:space="preserve">Block 3 — Linux primitives</t>
   </si>
   <si>
     <t xml:space="preserve">26 Oct–1 Nov</t>
@@ -186,7 +186,7 @@
     <t xml:space="preserve">Handshake, FIN and RST.</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 4 — proxies, TLS, timeouts</t>
+    <t xml:space="preserve">Block 4 — proxies, TLS, timeouts</t>
   </si>
   <si>
     <t xml:space="preserve">2–8 Nov</t>
@@ -219,7 +219,7 @@
     <t xml:space="preserve">Where timeouts come from.</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 5 — failure drills</t>
+    <t xml:space="preserve">Block 5 — failure drills</t>
   </si>
   <si>
     <t xml:space="preserve">9–15 Nov</t>
@@ -228,7 +228,7 @@
     <t xml:space="preserve">Reread it before the drills.</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 6 — security</t>
+    <t xml:space="preserve">Block 6 — security</t>
   </si>
   <si>
     <t xml:space="preserve">16–22 Nov</t>
@@ -243,7 +243,7 @@
     <t xml:space="preserve">Vocabulary for the threat model.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sections to skip until v1.0 (30 Nov 2026)</t>
+    <t xml:space="preserve">Sections to skip until v1.0 (30 Dec 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Topic</t>
@@ -345,7 +345,7 @@
     <t xml:space="preserve">Save for after v1.0</t>
   </si>
   <si>
-    <t xml:space="preserve">The plan excludes Azure work before 30 Nov. Useful later: (1) when you work through the plan's Azure mapping section, once routes, NSG-style filtering, private DNS and NAT are things you've built and captured yourself; (2) if you target roles where Azure infrastructure is part of the job.</t>
+    <t xml:space="preserve">The plan excludes Azure work before v1.0 ships. Useful later: (1) when you work through the plan's Azure mapping section, once routes, NSG-style filtering, private DNS and NAT are things you've built and captured yourself; (2) if you target roles where Azure infrastructure is part of the job.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources</t>
@@ -861,16 +861,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -888,29 +887,28 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="n">
-        <f aca="false">COUNTIF(F9:F24,"Read")</f>
+        <f aca="false">COUNTIF(E9:E24,"Read")</f>
         <v>0</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="n">
-        <f aca="false">COUNTA(C9:C24)</f>
+        <f aca="false">COUNTA(B9:B24)</f>
         <v>16</v>
       </c>
     </row>
@@ -928,21 +926,18 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="6" t="s">
         <v>12</v>
       </c>
     </row>
@@ -950,354 +945,306 @@
       <c r="A9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="9" t="s">
+      <c r="B9" s="9" t="s">
         <v>15</v>
       </c>
+      <c r="C9" s="8" t="s">
+        <v>16</v>
+      </c>
       <c r="D9" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="10"/>
+      <c r="E9" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="9" t="s">
+      <c r="B10" s="9" t="s">
         <v>21</v>
       </c>
+      <c r="C10" s="8" t="s">
+        <v>22</v>
+      </c>
       <c r="D10" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="10"/>
+      <c r="E10" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="9" t="s">
+      <c r="B11" s="9" t="s">
         <v>24</v>
       </c>
+      <c r="C11" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="D11" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="10"/>
+      <c r="E11" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="9" t="s">
+      <c r="B12" s="9" t="s">
         <v>27</v>
       </c>
+      <c r="C12" s="8" t="s">
+        <v>28</v>
+      </c>
       <c r="D12" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="10"/>
+      <c r="E12" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="9" t="s">
+      <c r="B13" s="9" t="s">
         <v>30</v>
       </c>
+      <c r="C13" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="D13" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="10"/>
+      <c r="E13" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="9" t="s">
+      <c r="B14" s="9" t="s">
         <v>33</v>
       </c>
+      <c r="C14" s="8" t="s">
+        <v>34</v>
+      </c>
       <c r="D14" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="10"/>
+      <c r="E14" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="9" t="s">
+      <c r="B15" s="9" t="s">
         <v>38</v>
       </c>
+      <c r="C15" s="8" t="s">
+        <v>39</v>
+      </c>
       <c r="D15" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="10"/>
+      <c r="E15" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="9" t="s">
+      <c r="B16" s="9" t="s">
         <v>41</v>
       </c>
+      <c r="C16" s="8" t="s">
+        <v>42</v>
+      </c>
       <c r="D16" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" s="10"/>
+      <c r="E16" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="9" t="s">
+      <c r="B17" s="9" t="s">
         <v>44</v>
       </c>
+      <c r="C17" s="8" t="s">
+        <v>45</v>
+      </c>
       <c r="D17" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G17" s="10"/>
+      <c r="E17" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" s="9" t="s">
+      <c r="B18" s="9" t="s">
         <v>47</v>
       </c>
+      <c r="C18" s="8" t="s">
+        <v>48</v>
+      </c>
       <c r="D18" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E18" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G18" s="10"/>
+      <c r="E18" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="9" t="s">
+      <c r="B19" s="9" t="s">
         <v>50</v>
       </c>
+      <c r="C19" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="D19" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="E19" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G19" s="10"/>
+      <c r="E19" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="9" t="s">
+      <c r="B20" s="9" t="s">
         <v>55</v>
       </c>
+      <c r="C20" s="8" t="s">
+        <v>56</v>
+      </c>
       <c r="D20" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G20" s="10"/>
+      <c r="E20" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="9" t="s">
+      <c r="B21" s="9" t="s">
         <v>58</v>
       </c>
+      <c r="C21" s="8" t="s">
+        <v>59</v>
+      </c>
       <c r="D21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E21" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="F21" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G21" s="10"/>
+      <c r="E21" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="9" t="s">
+      <c r="B22" s="9" t="s">
         <v>61</v>
       </c>
+      <c r="C22" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="D22" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="E22" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G22" s="10"/>
+      <c r="E22" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" s="9" t="s">
+      <c r="B23" s="9" t="s">
         <v>33</v>
       </c>
+      <c r="C23" s="8" t="s">
+        <v>34</v>
+      </c>
       <c r="D23" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E23" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G23" s="10"/>
+      <c r="E23" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C24" s="9" t="s">
+      <c r="B24" s="9" t="s">
         <v>69</v>
       </c>
+      <c r="C24" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="D24" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="E24" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="F24" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G24" s="10"/>
+      <c r="E24" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A8:G24"/>
+  <autoFilter ref="A8:F24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="C4:F4"/>
   </mergeCells>
-  <conditionalFormatting sqref="A9:G24">
+  <conditionalFormatting sqref="A9:F24">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
-      <formula>$F9="Read"</formula>
+      <formula>$E9="Read"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
-      <formula>$F9="Reading"</formula>
+      <formula>$E9="Reading"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" error="Choose Not read, Reading or Read." errorStyle="stop" errorTitle="Invalid status" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F9:F24" type="list">
+    <dataValidation allowBlank="false" error="Choose Not read, Reading or Read." errorStyle="stop" errorTitle="Invalid status" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E9:E24" type="list">
       <formula1>"Not read,Reading,Read"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>